<commit_message>
Fix country ref and lon/lat iun nodes.xlsx
</commit_message>
<xml_diff>
--- a/dac_offshore/clean_data/nodes/nodes.xlsx
+++ b/dac_offshore/clean_data/nodes/nodes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwiegner\PycharmProjects\AdOpT_DAC-Offshore\dac_offshore\clean_data\nodes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B29B458-7F62-4A80-8B55-A562674EE22B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D54304-BE54-40EE-B7D9-95D682F338E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-1965" windowWidth="21840" windowHeight="37920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2040" sheetId="1" r:id="rId1"/>
@@ -629,10 +629,10 @@
         <v>51</v>
       </c>
       <c r="D2">
-        <v>2.4529999999999998</v>
+        <v>2.89</v>
       </c>
       <c r="E2">
-        <v>51.496000000000002</v>
+        <v>51.612000000000002</v>
       </c>
       <c r="F2">
         <v>10598664.166826677</v>
@@ -649,13 +649,13 @@
         <v>44</v>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D3">
-        <v>2.89</v>
+        <v>6.1130000000000004</v>
       </c>
       <c r="E3">
-        <v>51.612000000000002</v>
+        <v>54.387999999999998</v>
       </c>
       <c r="F3">
         <v>14337830.405418999</v>
@@ -672,13 +672,13 @@
         <v>44</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D4">
-        <v>3.056</v>
+        <v>6.5910000000000002</v>
       </c>
       <c r="E4">
-        <v>51.011000000000003</v>
+        <v>54.021999999999998</v>
       </c>
       <c r="F4">
         <v>20187832.901575316</v>
@@ -695,13 +695,13 @@
         <v>44</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D5">
-        <v>4.8520000000000003</v>
+        <v>7.6970000000000001</v>
       </c>
       <c r="E5">
-        <v>50.595999999999997</v>
+        <v>54.453000000000003</v>
       </c>
       <c r="F5">
         <v>6634374.7998805381</v>
@@ -721,10 +721,10 @@
         <v>52</v>
       </c>
       <c r="D6">
-        <v>6.4409999999999998</v>
+        <v>7.21</v>
       </c>
       <c r="E6">
-        <v>54.177</v>
+        <v>55.131999999999998</v>
       </c>
       <c r="F6">
         <v>4900864.0276038777</v>
@@ -741,13 +741,13 @@
         <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D7">
-        <v>6.0330000000000004</v>
+        <v>7.7460000000000004</v>
       </c>
       <c r="E7">
-        <v>54.66</v>
+        <v>55.750999999999998</v>
       </c>
       <c r="F7">
         <v>5132008.3416757006</v>
@@ -764,13 +764,13 @@
         <v>44</v>
       </c>
       <c r="C8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D8">
-        <v>6.1130000000000004</v>
+        <v>2.99</v>
       </c>
       <c r="E8">
-        <v>54.387999999999998</v>
+        <v>51.698</v>
       </c>
       <c r="F8">
         <v>7967354.6775069907</v>
@@ -787,13 +787,13 @@
         <v>44</v>
       </c>
       <c r="C9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D9">
-        <v>6.5910000000000002</v>
+        <v>4.01</v>
       </c>
       <c r="E9">
-        <v>54.021999999999998</v>
+        <v>52.518999999999998</v>
       </c>
       <c r="F9">
         <v>21499911.3527757</v>
@@ -810,13 +810,13 @@
         <v>44</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D10">
-        <v>7.6970000000000001</v>
+        <v>5.9640000000000004</v>
       </c>
       <c r="E10">
-        <v>54.453000000000003</v>
+        <v>54.036000000000001</v>
       </c>
       <c r="F10">
         <v>3410422.0728563438</v>
@@ -833,13 +833,13 @@
         <v>44</v>
       </c>
       <c r="C11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D11">
-        <v>7.21</v>
+        <v>2.4529999999999998</v>
       </c>
       <c r="E11">
-        <v>55.131999999999998</v>
+        <v>51.496000000000002</v>
       </c>
       <c r="F11">
         <v>8630475.4178542346</v>
@@ -859,10 +859,10 @@
         <v>52</v>
       </c>
       <c r="D12">
-        <v>6.9630000000000001</v>
+        <v>6.4409999999999998</v>
       </c>
       <c r="E12">
-        <v>51.387</v>
+        <v>54.177</v>
       </c>
       <c r="F12">
         <v>9501057.1457648855</v>
@@ -882,10 +882,10 @@
         <v>52</v>
       </c>
       <c r="D13">
-        <v>7.8</v>
+        <v>6.0330000000000004</v>
       </c>
       <c r="E13">
-        <v>52.947000000000003</v>
+        <v>54.66</v>
       </c>
       <c r="F13">
         <v>39898912.306736194</v>
@@ -902,13 +902,13 @@
         <v>44</v>
       </c>
       <c r="C14" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D14">
-        <v>9.8059999999999992</v>
+        <v>7.6520000000000001</v>
       </c>
       <c r="E14">
-        <v>53.68</v>
+        <v>56.326000000000001</v>
       </c>
       <c r="F14">
         <v>2849903.799813719</v>
@@ -925,13 +925,13 @@
         <v>44</v>
       </c>
       <c r="C15" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D15">
-        <v>10.785</v>
+        <v>3.6080000000000001</v>
       </c>
       <c r="E15">
-        <v>50.637</v>
+        <v>52.927999999999997</v>
       </c>
       <c r="F15">
         <v>15922855.977153704</v>
@@ -948,13 +948,13 @@
         <v>44</v>
       </c>
       <c r="C16" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="D16">
-        <v>7.6520000000000001</v>
+        <v>3.1779999999999999</v>
       </c>
       <c r="E16">
-        <v>56.326000000000001</v>
+        <v>53.1</v>
       </c>
       <c r="F16">
         <v>5398087.0600787401</v>
@@ -971,13 +971,13 @@
         <v>44</v>
       </c>
       <c r="C17" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="D17">
-        <v>7.7460000000000004</v>
+        <v>1.1679999999999999</v>
       </c>
       <c r="E17">
-        <v>55.750999999999998</v>
+        <v>53.49</v>
       </c>
       <c r="F17">
         <v>15405100.552037166</v>
@@ -994,13 +994,13 @@
         <v>44</v>
       </c>
       <c r="C18" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="D18">
-        <v>10.051</v>
+        <v>2.0179999999999998</v>
       </c>
       <c r="E18">
-        <v>55.959000000000003</v>
+        <v>54.834000000000003</v>
       </c>
       <c r="F18">
         <v>22717804.839875247</v>
@@ -1017,13 +1017,13 @@
         <v>44</v>
       </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D19">
-        <v>3.6080000000000001</v>
+        <v>-1.734</v>
       </c>
       <c r="E19">
-        <v>52.927999999999997</v>
+        <v>56.383000000000003</v>
       </c>
       <c r="F19">
         <v>22584182.924791206</v>
@@ -1040,13 +1040,13 @@
         <v>44</v>
       </c>
       <c r="C20" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D20">
-        <v>3.1779999999999999</v>
+        <v>-2.7069999999999999</v>
       </c>
       <c r="E20">
-        <v>53.1</v>
+        <v>58.180999999999997</v>
       </c>
       <c r="F20">
         <v>15473456.469615718</v>
@@ -1063,13 +1063,13 @@
         <v>44</v>
       </c>
       <c r="C21" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D21">
-        <v>2.99</v>
+        <v>2.1259999999999999</v>
       </c>
       <c r="E21">
-        <v>51.698</v>
+        <v>53.896000000000001</v>
       </c>
       <c r="F21">
         <v>23543033.66675758</v>
@@ -1086,13 +1086,13 @@
         <v>44</v>
       </c>
       <c r="C22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D22">
-        <v>4.01</v>
+        <v>2.8380000000000001</v>
       </c>
       <c r="E22">
-        <v>52.518999999999998</v>
+        <v>52.908000000000001</v>
       </c>
       <c r="F22">
         <v>14719528.576583225</v>
@@ -1109,13 +1109,13 @@
         <v>44</v>
       </c>
       <c r="C23" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D23">
-        <v>5.9640000000000004</v>
+        <v>2.2320000000000002</v>
       </c>
       <c r="E23">
-        <v>54.036000000000001</v>
+        <v>52.11</v>
       </c>
       <c r="F23">
         <v>13195804.086936183</v>
@@ -1132,13 +1132,13 @@
         <v>45</v>
       </c>
       <c r="C24" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D24">
-        <v>4.2439999999999998</v>
+        <v>-0.18099999999999999</v>
       </c>
       <c r="E24">
-        <v>51.761000000000003</v>
+        <v>60.304000000000002</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -1155,13 +1155,13 @@
         <v>45</v>
       </c>
       <c r="C25" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D25">
-        <v>4.9950000000000001</v>
+        <v>-5.0750000000000002</v>
       </c>
       <c r="E25">
-        <v>52.45</v>
+        <v>58.83</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -1178,13 +1178,13 @@
         <v>45</v>
       </c>
       <c r="C26" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D26">
-        <v>6.1239999999999997</v>
+        <v>-1.294</v>
       </c>
       <c r="E26">
-        <v>52.95</v>
+        <v>58.362000000000002</v>
       </c>
       <c r="F26">
         <v>0</v>
@@ -1201,13 +1201,13 @@
         <v>45</v>
       </c>
       <c r="C27" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D27">
-        <v>5.8019999999999996</v>
+        <v>-0.41799999999999998</v>
       </c>
       <c r="E27">
-        <v>51.866</v>
+        <v>57.009</v>
       </c>
       <c r="F27">
         <v>0</v>
@@ -1227,10 +1227,10 @@
         <v>49</v>
       </c>
       <c r="D28">
-        <v>7.5910000000000002</v>
+        <v>25.641999999999999</v>
       </c>
       <c r="E28">
-        <v>59.381999999999998</v>
+        <v>71.424999999999997</v>
       </c>
       <c r="F28">
         <v>0</v>
@@ -1247,13 +1247,13 @@
         <v>45</v>
       </c>
       <c r="C29" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D29">
-        <v>1.1679999999999999</v>
+        <v>7.7690000000000001</v>
       </c>
       <c r="E29">
-        <v>53.49</v>
+        <v>64.844999999999999</v>
       </c>
       <c r="F29">
         <v>0</v>
@@ -1270,13 +1270,13 @@
         <v>45</v>
       </c>
       <c r="C30" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D30">
-        <v>2.0179999999999998</v>
+        <v>4.1550000000000002</v>
       </c>
       <c r="E30">
-        <v>54.834000000000003</v>
+        <v>59.642000000000003</v>
       </c>
       <c r="F30">
         <v>0</v>
@@ -1293,13 +1293,13 @@
         <v>45</v>
       </c>
       <c r="C31" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D31">
-        <v>-1.734</v>
+        <v>4.8019999999999996</v>
       </c>
       <c r="E31">
-        <v>56.383000000000003</v>
+        <v>57.234999999999999</v>
       </c>
       <c r="F31">
         <v>0</v>
@@ -1316,13 +1316,13 @@
         <v>45</v>
       </c>
       <c r="C32" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D32">
-        <v>-2.7069999999999999</v>
+        <v>5.6420000000000003</v>
       </c>
       <c r="E32">
-        <v>58.180999999999997</v>
+        <v>54.021000000000001</v>
       </c>
       <c r="F32">
         <v>0</v>
@@ -1339,13 +1339,13 @@
         <v>45</v>
       </c>
       <c r="C33" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D33">
-        <v>0.69599999999999995</v>
+        <v>3.9359999999999999</v>
       </c>
       <c r="E33">
-        <v>52.103999999999999</v>
+        <v>53.177999999999997</v>
       </c>
       <c r="F33">
         <v>0</v>
@@ -1362,13 +1362,13 @@
         <v>45</v>
       </c>
       <c r="C34" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="D34">
-        <v>-1.6639999999999999</v>
+        <v>6.6260000000000003</v>
       </c>
       <c r="E34">
-        <v>53.993000000000002</v>
+        <v>56.265999999999998</v>
       </c>
       <c r="F34">
         <v>0</v>
@@ -1385,13 +1385,13 @@
         <v>45</v>
       </c>
       <c r="C35" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D35">
-        <v>-4.5810000000000004</v>
+        <v>3.637</v>
       </c>
       <c r="E35">
-        <v>56.476999999999997</v>
+        <v>55.784999999999997</v>
       </c>
       <c r="F35">
         <v>0</v>
@@ -1408,13 +1408,13 @@
         <v>45</v>
       </c>
       <c r="C36" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D36">
-        <v>-2.4449999999999998</v>
+        <v>5.0640000000000001</v>
       </c>
       <c r="E36">
-        <v>51.76</v>
+        <v>55.156999999999996</v>
       </c>
       <c r="F36">
         <v>0</v>
@@ -1431,13 +1431,13 @@
         <v>45</v>
       </c>
       <c r="C37" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D37">
-        <v>2.1259999999999999</v>
+        <v>6.3609999999999998</v>
       </c>
       <c r="E37">
-        <v>53.896000000000001</v>
+        <v>55.012</v>
       </c>
       <c r="F37">
         <v>0</v>
@@ -1454,13 +1454,13 @@
         <v>73</v>
       </c>
       <c r="C38" t="s">
-        <v>54</v>
-      </c>
-      <c r="D38">
-        <v>2.8380000000000001</v>
-      </c>
-      <c r="E38">
-        <v>52.908000000000001</v>
+        <v>47</v>
+      </c>
+      <c r="D38" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E38" t="e">
+        <v>#N/A</v>
       </c>
       <c r="F38">
         <v>0</v>
@@ -1477,13 +1477,13 @@
         <v>73</v>
       </c>
       <c r="C39" t="s">
-        <v>54</v>
-      </c>
-      <c r="D39">
-        <v>2.2320000000000002</v>
-      </c>
-      <c r="E39">
-        <v>52.11</v>
+        <v>49</v>
+      </c>
+      <c r="D39" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E39" t="e">
+        <v>#N/A</v>
       </c>
       <c r="F39">
         <v>0</v>
@@ -1500,13 +1500,13 @@
         <v>73</v>
       </c>
       <c r="C40" t="s">
-        <v>54</v>
-      </c>
-      <c r="D40">
-        <v>-0.18099999999999999</v>
-      </c>
-      <c r="E40">
-        <v>60.304000000000002</v>
+        <v>49</v>
+      </c>
+      <c r="D40" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E40" t="e">
+        <v>#N/A</v>
       </c>
       <c r="F40">
         <v>0</v>
@@ -1523,13 +1523,13 @@
         <v>18</v>
       </c>
       <c r="C41" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D41">
-        <v>-5.0750000000000002</v>
+        <v>3.056</v>
       </c>
       <c r="E41">
-        <v>58.83</v>
+        <v>51.011000000000003</v>
       </c>
       <c r="F41">
         <v>4043961.5764071145</v>
@@ -1546,13 +1546,13 @@
         <v>18</v>
       </c>
       <c r="C42" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D42">
-        <v>-1.294</v>
+        <v>4.8520000000000003</v>
       </c>
       <c r="E42">
-        <v>58.362000000000002</v>
+        <v>50.595999999999997</v>
       </c>
       <c r="F42">
         <v>21551858.554255962</v>
@@ -1569,13 +1569,13 @@
         <v>18</v>
       </c>
       <c r="C43" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D43">
-        <v>-0.41799999999999998</v>
+        <v>6.9630000000000001</v>
       </c>
       <c r="E43">
-        <v>57.009</v>
+        <v>51.387</v>
       </c>
       <c r="F43">
         <v>20503050.983261846</v>
@@ -1592,13 +1592,13 @@
         <v>18</v>
       </c>
       <c r="C44" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D44">
-        <v>25.641999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="E44">
-        <v>71.424999999999997</v>
+        <v>52.947000000000003</v>
       </c>
       <c r="F44">
         <v>25771359.031673171</v>
@@ -1615,13 +1615,13 @@
         <v>18</v>
       </c>
       <c r="C45" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D45">
-        <v>7.7690000000000001</v>
+        <v>9.8059999999999992</v>
       </c>
       <c r="E45">
-        <v>64.844999999999999</v>
+        <v>53.68</v>
       </c>
       <c r="F45">
         <v>47538734.794128776</v>
@@ -1638,13 +1638,13 @@
         <v>18</v>
       </c>
       <c r="C46" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D46">
-        <v>4.1550000000000002</v>
+        <v>10.785</v>
       </c>
       <c r="E46">
-        <v>59.642000000000003</v>
+        <v>50.637</v>
       </c>
       <c r="F46">
         <v>227466324.89891711</v>
@@ -1661,13 +1661,13 @@
         <v>18</v>
       </c>
       <c r="C47" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D47">
-        <v>4.8019999999999996</v>
+        <v>10.051</v>
       </c>
       <c r="E47">
-        <v>57.234999999999999</v>
+        <v>55.959000000000003</v>
       </c>
       <c r="F47">
         <v>52181755.753615983</v>
@@ -1687,10 +1687,10 @@
         <v>53</v>
       </c>
       <c r="D48">
-        <v>5.6420000000000003</v>
+        <v>4.2439999999999998</v>
       </c>
       <c r="E48">
-        <v>54.021000000000001</v>
+        <v>51.761000000000003</v>
       </c>
       <c r="F48">
         <v>9154220.897037236</v>
@@ -1710,10 +1710,10 @@
         <v>53</v>
       </c>
       <c r="D49">
-        <v>3.9359999999999999</v>
+        <v>4.9950000000000001</v>
       </c>
       <c r="E49">
-        <v>53.177999999999997</v>
+        <v>52.45</v>
       </c>
       <c r="F49">
         <v>8263128.149645159</v>
@@ -1730,13 +1730,13 @@
         <v>18</v>
       </c>
       <c r="C50" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="D50">
-        <v>6.6260000000000003</v>
+        <v>6.1239999999999997</v>
       </c>
       <c r="E50">
-        <v>56.265999999999998</v>
+        <v>52.95</v>
       </c>
       <c r="F50">
         <v>24106078.277672008</v>
@@ -1753,13 +1753,13 @@
         <v>18</v>
       </c>
       <c r="C51" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D51">
-        <v>3.637</v>
+        <v>5.8019999999999996</v>
       </c>
       <c r="E51">
-        <v>55.784999999999997</v>
+        <v>51.866</v>
       </c>
       <c r="F51">
         <v>14416688.836987048</v>
@@ -1776,13 +1776,13 @@
         <v>18</v>
       </c>
       <c r="C52" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D52">
-        <v>5.0640000000000001</v>
+        <v>7.5910000000000002</v>
       </c>
       <c r="E52">
-        <v>55.156999999999996</v>
+        <v>59.381999999999998</v>
       </c>
       <c r="F52">
         <v>21306749.86132694</v>
@@ -1799,13 +1799,13 @@
         <v>18</v>
       </c>
       <c r="C53" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D53">
-        <v>6.3609999999999998</v>
+        <v>0.69599999999999995</v>
       </c>
       <c r="E53">
-        <v>55.012</v>
+        <v>52.103999999999999</v>
       </c>
       <c r="F53">
         <v>16551362.594586601</v>
@@ -1822,13 +1822,13 @@
         <v>18</v>
       </c>
       <c r="C54" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="D54">
-        <v>4.67</v>
+        <v>-1.6639999999999999</v>
       </c>
       <c r="E54">
-        <v>56.35</v>
+        <v>53.993000000000002</v>
       </c>
       <c r="F54">
         <v>56740997.686032154</v>
@@ -1845,13 +1845,13 @@
         <v>18</v>
       </c>
       <c r="C55" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D55">
-        <v>3.16</v>
+        <v>-4.5810000000000004</v>
       </c>
       <c r="E55">
-        <v>60.46</v>
+        <v>56.476999999999997</v>
       </c>
       <c r="F55">
         <v>46042938.052974679</v>
@@ -1868,13 +1868,13 @@
         <v>18</v>
       </c>
       <c r="C56" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D56">
-        <v>1.9</v>
+        <v>-2.4449999999999998</v>
       </c>
       <c r="E56">
-        <v>58.35</v>
+        <v>51.76</v>
       </c>
       <c r="F56">
         <v>47118700.601414301</v>

</xml_diff>